<commit_message>
Regenerate CNA recert binder package
</commit_message>
<xml_diff>
--- a/CNA-Recert-Course/_CNA_Recert/CNA-Recert-Course_CNA_Recert/CNA_Recertification_Executive_Task_Tracker.xlsx
+++ b/CNA-Recert-Course/_CNA_Recert/CNA-Recert-Course_CNA_Recert/CNA_Recertification_Executive_Task_Tracker.xlsx
@@ -25801,47 +25801,47 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>P0 Blocker</t>
+          <t>P1 High</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>Needs Source Repair</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>Resolve CCCCO/source repair evidence</t>
+          <t>Maintain NATP 10-17 source evidence</t>
         </is>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
-          <t>Survey evidence + ContentV2 gaps</t>
+          <t>Survey evidence + ContentV2 maps</t>
         </is>
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>72 mapped objectives; 7 source repair</t>
+          <t>72 mapped objectives; 0 source repair; 0 SME review</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>Unresolved CCCCO gaps</t>
+          <t>Evidence drift</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr">
         <is>
-          <t>Repair M03 and under-depth objectives</t>
+          <t>Re-run validation after source changes</t>
         </is>
       </c>
       <c r="L202" s="2" t="inlineStr">
@@ -25851,7 +25851,7 @@
       </c>
       <c r="M202" s="2" t="inlineStr">
         <is>
-          <t>SME</t>
+          <t>Compliance</t>
         </is>
       </c>
       <c r="N202" s="2" t="inlineStr">
@@ -25899,7 +25899,7 @@
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>Needs Compliance Review</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F203" s="2" t="inlineStr">
@@ -25909,7 +25909,7 @@
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>Close time-depth gap with source-backed expansion</t>
+          <t>Preserve 720-minute normalized time model</t>
         </is>
       </c>
       <c r="H203" s="2" t="inlineStr">
@@ -25919,17 +25919,17 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>447.12 active-learning min estimate</t>
+          <t>782.73 active-learning min estimate; 0 failing lessons</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>Under-depth lessons</t>
+          <t>Active-time method not yet approved</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
         <is>
-          <t>Expand without padding</t>
+          <t>Keep audit in sync and validate active-time method</t>
         </is>
       </c>
       <c r="L203" s="2" t="inlineStr">
@@ -25944,7 +25944,7 @@
       </c>
       <c r="N203" s="2" t="inlineStr">
         <is>
-          <t>Source Evidence</t>
+          <t>ContentV2</t>
         </is>
       </c>
       <c r="O203" s="2" t="inlineStr">
@@ -25987,7 +25987,7 @@
       </c>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>Needs SME Review</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F204" s="2" t="inlineStr">
@@ -30652,47 +30652,47 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>P0 Blocker</t>
+          <t>P1 High</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>Needs Source Repair</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>Resolve CCCCO/source repair evidence</t>
+          <t>Maintain NATP 10-17 source evidence</t>
         </is>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
-          <t>Survey evidence + ContentV2 gaps</t>
+          <t>Survey evidence + ContentV2 maps</t>
         </is>
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>72 mapped objectives; 7 source repair</t>
+          <t>72 mapped objectives; 0 source repair; 0 SME review</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>Unresolved CCCCO gaps</t>
+          <t>Evidence drift</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr">
         <is>
-          <t>Repair M03 and under-depth objectives</t>
+          <t>Re-run validation after source changes</t>
         </is>
       </c>
       <c r="L202" s="2" t="inlineStr">
@@ -30702,7 +30702,7 @@
       </c>
       <c r="M202" s="2" t="inlineStr">
         <is>
-          <t>SME</t>
+          <t>Compliance</t>
         </is>
       </c>
       <c r="N202" s="2" t="inlineStr">
@@ -30750,7 +30750,7 @@
       </c>
       <c r="E203" s="2" t="inlineStr">
         <is>
-          <t>Needs Compliance Review</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F203" s="2" t="inlineStr">
@@ -30760,7 +30760,7 @@
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>Close time-depth gap with source-backed expansion</t>
+          <t>Preserve 720-minute normalized time model</t>
         </is>
       </c>
       <c r="H203" s="2" t="inlineStr">
@@ -30770,17 +30770,17 @@
       </c>
       <c r="I203" s="2" t="inlineStr">
         <is>
-          <t>447.12 active-learning min estimate</t>
+          <t>782.73 active-learning min estimate; 0 failing lessons</t>
         </is>
       </c>
       <c r="J203" s="2" t="inlineStr">
         <is>
-          <t>Under-depth lessons</t>
+          <t>Active-time method not yet approved</t>
         </is>
       </c>
       <c r="K203" s="2" t="inlineStr">
         <is>
-          <t>Expand without padding</t>
+          <t>Keep audit in sync and validate active-time method</t>
         </is>
       </c>
       <c r="L203" s="2" t="inlineStr">
@@ -30795,7 +30795,7 @@
       </c>
       <c r="N203" s="2" t="inlineStr">
         <is>
-          <t>Source Evidence</t>
+          <t>ContentV2</t>
         </is>
       </c>
       <c r="O203" s="2" t="inlineStr">
@@ -30838,7 +30838,7 @@
       </c>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>Needs SME Review</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F204" s="2" t="inlineStr">
@@ -31379,7 +31379,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R210"/>
+  <dimension ref="A1:R211"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -35568,17 +35568,17 @@
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
-          <t>Unified Blueprint; Content syllabus</t>
+          <t>Orientation/compliance exception</t>
         </is>
       </c>
       <c r="G203" s="2" t="inlineStr">
         <is>
-          <t>Legal/CDPH copy review</t>
+          <t>Compliance/legal review before production</t>
         </is>
       </c>
       <c r="H203" s="2" t="inlineStr">
         <is>
-          <t>Confirm acknowledgements and no-PHI language</t>
+          <t>Use for Package A, Package B, and custom Package C</t>
         </is>
       </c>
       <c r="I203" s="2" t="n"/>
@@ -35595,40 +35595,40 @@
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
         <is>
-          <t>M01</t>
+          <t>M10</t>
         </is>
       </c>
       <c r="B204" s="2" t="inlineStr">
         <is>
-          <t>Infection Control and PPE</t>
+          <t>NATP Module 10: Vital Signs</t>
         </is>
       </c>
       <c r="C204" s="2" t="n">
-        <v>90</v>
+        <v>83</v>
       </c>
       <c r="D204" s="2" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>17</t>
         </is>
       </c>
       <c r="E204" s="2" t="inlineStr">
         <is>
-          <t>Needs SME Review</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
-          <t>Legacy CNA-CE draft + scattered CCCCO refs</t>
+          <t>NATP Module 10</t>
         </is>
       </c>
       <c r="G204" s="2" t="inlineStr">
         <is>
-          <t>No dedicated NATP 10-17 source</t>
+          <t>None identified</t>
         </is>
       </c>
       <c r="H204" s="2" t="inlineStr">
         <is>
-          <t>SME/source review and source-backed expansion</t>
+          <t>Maintain source-backed coverage</t>
         </is>
       </c>
       <c r="I204" s="2" t="n"/>
@@ -35645,40 +35645,40 @@
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
         <is>
-          <t>M02</t>
+          <t>M11</t>
         </is>
       </c>
       <c r="B205" s="2" t="inlineStr">
         <is>
-          <t>Resident Rights, Abuse Prevention, and Boundaries</t>
+          <t>NATP Module 11: Nutrition</t>
         </is>
       </c>
       <c r="C205" s="2" t="n">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="D205" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E205" s="2" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
-          <t>CCCCO/NATP Module 17</t>
+          <t>NATP Module 11</t>
         </is>
       </c>
       <c r="G205" s="2" t="inlineStr">
         <is>
-          <t>Under-depth expansion</t>
+          <t>None identified</t>
         </is>
       </c>
       <c r="H205" s="2" t="inlineStr">
         <is>
-          <t>Expand partial objectives from source</t>
+          <t>Maintain source-backed coverage</t>
         </is>
       </c>
       <c r="I205" s="2" t="n"/>
@@ -35695,40 +35695,40 @@
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
         <is>
-          <t>M03</t>
+          <t>M12</t>
         </is>
       </c>
       <c r="B206" s="2" t="inlineStr">
         <is>
-          <t>Dementia, Communication, and Respectful Care</t>
+          <t>NATP Module 12: Emergency Procedures</t>
         </is>
       </c>
       <c r="C206" s="2" t="n">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="D206" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E206" s="2" t="inlineStr">
         <is>
-          <t>Needs Source Repair</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
-          <t>CCCCO/NATP Modules 13, 16</t>
+          <t>NATP Module 12</t>
         </is>
       </c>
       <c r="G206" s="2" t="inlineStr">
         <is>
-          <t>Sensitive content and truncated source</t>
+          <t>None identified</t>
         </is>
       </c>
       <c r="H206" s="2" t="inlineStr">
         <is>
-          <t>Repair M03/L03-L05 from CCCCO M16 and SME review</t>
+          <t>Maintain source-backed coverage</t>
         </is>
       </c>
       <c r="I206" s="2" t="n"/>
@@ -35745,40 +35745,40 @@
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
         <is>
-          <t>M04</t>
+          <t>M13</t>
         </is>
       </c>
       <c r="B207" s="2" t="inlineStr">
         <is>
-          <t>Mobility, Falls, and Workplace Safety</t>
+          <t>NATP Module 13: Long Term Care Resident</t>
         </is>
       </c>
       <c r="C207" s="2" t="n">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="D207" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>16</t>
         </is>
       </c>
       <c r="E207" s="2" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
-          <t>CCCCO/NATP Modules 12, 14</t>
+          <t>NATP Module 13</t>
         </is>
       </c>
       <c r="G207" s="2" t="inlineStr">
         <is>
-          <t>No hands-on competency claim</t>
+          <t>None identified</t>
         </is>
       </c>
       <c r="H207" s="2" t="inlineStr">
         <is>
-          <t>Expand source-backed safety/restorative content</t>
+          <t>Maintain source-backed coverage</t>
         </is>
       </c>
       <c r="I207" s="2" t="n"/>
@@ -35795,40 +35795,40 @@
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
         <is>
-          <t>M05</t>
+          <t>M14</t>
         </is>
       </c>
       <c r="B208" s="2" t="inlineStr">
         <is>
-          <t>Nutrition, Skin Integrity, Vital Signs</t>
+          <t>NATP Module 14: Rehabilitative Nursing</t>
         </is>
       </c>
       <c r="C208" s="2" t="n">
-        <v>120</v>
+        <v>55</v>
       </c>
       <c r="D208" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E208" s="2" t="inlineStr">
         <is>
-          <t>Needs SME Review</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
-          <t>CCCCO/NATP Modules 10, 11, 13</t>
+          <t>NATP Module 14</t>
         </is>
       </c>
       <c r="G208" s="2" t="inlineStr">
         <is>
-          <t>Pressure-injury scope review</t>
+          <t>None identified</t>
         </is>
       </c>
       <c r="H208" s="2" t="inlineStr">
         <is>
-          <t>SME review and CNA-scope wording check</t>
+          <t>Maintain source-backed coverage</t>
         </is>
       </c>
       <c r="I208" s="2" t="n"/>
@@ -35845,40 +35845,40 @@
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
         <is>
-          <t>M06</t>
+          <t>M15</t>
         </is>
       </c>
       <c r="B209" s="2" t="inlineStr">
         <is>
-          <t>Documentation, Reporting, PHI Avoidance, and Scope</t>
+          <t>NATP Module 15: Observation and Charting</t>
         </is>
       </c>
       <c r="C209" s="2" t="n">
-        <v>90</v>
+        <v>111</v>
       </c>
       <c r="D209" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="E209" s="2" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
-          <t>CCCCO/NATP Module 15</t>
+          <t>NATP Module 15</t>
         </is>
       </c>
       <c r="G209" s="2" t="inlineStr">
         <is>
-          <t>PHI and scope controls</t>
+          <t>None identified</t>
         </is>
       </c>
       <c r="H209" s="2" t="inlineStr">
         <is>
-          <t>Confirm no PHI free text and expand source-backed content</t>
+          <t>Maintain source-backed coverage</t>
         </is>
       </c>
       <c r="I209" s="2" t="n"/>
@@ -35895,40 +35895,40 @@
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
         <is>
-          <t>M07</t>
+          <t>M16</t>
         </is>
       </c>
       <c r="B210" s="2" t="inlineStr">
         <is>
-          <t>Final Review, Exam/Test, Affidavit</t>
+          <t>NATP Module 16: Death and Dying</t>
         </is>
       </c>
       <c r="C210" s="2" t="n">
-        <v>30</v>
+        <v>55</v>
       </c>
       <c r="D210" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E210" s="2" t="inlineStr">
         <is>
-          <t>Needs Legal/CDPH Review</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
-          <t>All modules; final assessment map</t>
+          <t>NATP Module 16</t>
         </is>
       </c>
       <c r="G210" s="2" t="inlineStr">
         <is>
-          <t>Affidavit/certificate approval</t>
+          <t>None identified</t>
         </is>
       </c>
       <c r="H210" s="2" t="inlineStr">
         <is>
-          <t>Approve final wording and keep certificate disabled</t>
+          <t>Maintain source-backed coverage</t>
         </is>
       </c>
       <c r="I210" s="2" t="n"/>
@@ -35942,9 +35942,59 @@
       <c r="Q210" s="2" t="n"/>
       <c r="R210" s="2" t="n"/>
     </row>
+    <row r="211">
+      <c r="A211" s="2" t="inlineStr">
+        <is>
+          <t>M17</t>
+        </is>
+      </c>
+      <c r="B211" s="2" t="inlineStr">
+        <is>
+          <t>NATP Module 17: Patient/Resident Abuse</t>
+        </is>
+      </c>
+      <c r="C211" s="2" t="n">
+        <v>168</v>
+      </c>
+      <c r="D211" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E211" s="2" t="inlineStr">
+        <is>
+          <t>Drafted</t>
+        </is>
+      </c>
+      <c r="F211" s="2" t="inlineStr">
+        <is>
+          <t>NATP Module 17</t>
+        </is>
+      </c>
+      <c r="G211" s="2" t="inlineStr">
+        <is>
+          <t>None identified</t>
+        </is>
+      </c>
+      <c r="H211" s="2" t="inlineStr">
+        <is>
+          <t>Maintain source-backed coverage</t>
+        </is>
+      </c>
+      <c r="I211" s="2" t="n"/>
+      <c r="J211" s="2" t="n"/>
+      <c r="K211" s="2" t="n"/>
+      <c r="L211" s="2" t="n"/>
+      <c r="M211" s="2" t="n"/>
+      <c r="N211" s="2" t="n"/>
+      <c r="O211" s="2" t="n"/>
+      <c r="P211" s="2" t="n"/>
+      <c r="Q211" s="2" t="n"/>
+      <c r="R211" s="2" t="n"/>
+    </row>
   </sheetData>
   <autoFilter ref="A1:R9"/>
-  <conditionalFormatting sqref="E2:E210">
+  <conditionalFormatting sqref="E2:E211">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>ISNUMBER(SEARCH("Blocked",E2))</formula>
     </cfRule>
@@ -35955,7 +36005,7 @@
       <formula>E2="Complete"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="C2:C210">
+  <conditionalFormatting sqref="C2:C211">
     <cfRule type="expression" priority="4" dxfId="0">
       <formula>ISNUMBER(SEARCH("P0",C2))</formula>
     </cfRule>
@@ -40102,47 +40152,47 @@
       </c>
       <c r="C202" s="2" t="inlineStr">
         <is>
-          <t>P0 Blocker</t>
+          <t>P1 High</t>
         </is>
       </c>
       <c r="D202" s="2" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Medium</t>
         </is>
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>Needs Source Repair</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>Resolve CCCCO/source repair evidence</t>
+          <t>Maintain NATP 10-17 source evidence</t>
         </is>
       </c>
       <c r="H202" s="2" t="inlineStr">
         <is>
-          <t>Survey evidence + ContentV2 gaps</t>
+          <t>Survey evidence + ContentV2 maps</t>
         </is>
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>72 mapped objectives; 7 source repair</t>
+          <t>72 mapped objectives; 0 source repair; 0 SME review</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>Unresolved CCCCO gaps</t>
+          <t>Evidence drift</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr">
         <is>
-          <t>Repair M03 and under-depth objectives</t>
+          <t>Re-run validation after source changes</t>
         </is>
       </c>
       <c r="L202" s="2" t="inlineStr">
@@ -40152,7 +40202,7 @@
       </c>
       <c r="M202" s="2" t="inlineStr">
         <is>
-          <t>SME</t>
+          <t>Compliance</t>
         </is>
       </c>
       <c r="N202" s="2" t="inlineStr">
@@ -44347,7 +44397,7 @@
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>Needs Compliance Review</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F202" s="2" t="inlineStr">
@@ -44357,7 +44407,7 @@
       </c>
       <c r="G202" s="2" t="inlineStr">
         <is>
-          <t>Close time-depth gap with source-backed expansion</t>
+          <t>Preserve 720-minute normalized time model</t>
         </is>
       </c>
       <c r="H202" s="2" t="inlineStr">
@@ -44367,17 +44417,17 @@
       </c>
       <c r="I202" s="2" t="inlineStr">
         <is>
-          <t>447.12 active-learning min estimate</t>
+          <t>782.73 active-learning min estimate; 0 failing lessons</t>
         </is>
       </c>
       <c r="J202" s="2" t="inlineStr">
         <is>
-          <t>Under-depth lessons</t>
+          <t>Active-time method not yet approved</t>
         </is>
       </c>
       <c r="K202" s="2" t="inlineStr">
         <is>
-          <t>Expand without padding</t>
+          <t>Keep audit in sync and validate active-time method</t>
         </is>
       </c>
       <c r="L202" s="2" t="inlineStr">
@@ -44392,7 +44442,7 @@
       </c>
       <c r="N202" s="2" t="inlineStr">
         <is>
-          <t>Source Evidence</t>
+          <t>ContentV2</t>
         </is>
       </c>
       <c r="O202" s="2" t="inlineStr">
@@ -48582,7 +48632,7 @@
       </c>
       <c r="E202" s="2" t="inlineStr">
         <is>
-          <t>Needs SME Review</t>
+          <t>Drafted</t>
         </is>
       </c>
       <c r="F202" s="2" t="inlineStr">

</xml_diff>